<commit_message>
Perbaiki tampilna admin dan guru bidang studi
</commit_message>
<xml_diff>
--- a/server/public/templates/template_import_siswa.xlsx
+++ b/server/public/templates/template_import_siswa.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\E-Rapor_PBL\server\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\E-Rapor\server\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9007C017-4B9D-4056-BECA-13D9D143C63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E3C3630-1144-4920-A788-1C578E6CD8FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2892" yWindow="2892" windowWidth="17280" windowHeight="9420" xr2:uid="{64C7BB62-96F4-434D-B995-5E80C48BB89C}"/>
+    <workbookView xWindow="2472" yWindow="2472" windowWidth="17280" windowHeight="9420" xr2:uid="{64C7BB62-96F4-434D-B995-5E80C48BB89C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>nis</t>
   </si>
@@ -47,9 +47,6 @@
     <t>nama_lengkap</t>
   </si>
   <si>
-    <t>kelas_id</t>
-  </si>
-  <si>
     <t>tanggal_lahir</t>
   </si>
   <si>
@@ -65,9 +62,6 @@
     <t>21-2345</t>
   </si>
   <si>
-    <t>0012345678</t>
-  </si>
-  <si>
     <t>Mark</t>
   </si>
   <si>
@@ -81,9 +75,6 @@
   </si>
   <si>
     <t>Batu Aji</t>
-  </si>
-  <si>
-    <t>1 A</t>
   </si>
 </sst>
 </file>
@@ -473,68 +464,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F0188A5-9EC4-4B4E-B85A-6FC24964397F}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="12.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="11.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="3">
+        <v>12345678</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>12</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>